<commit_message>
Agregar interfaz interactiva, sistema de recomendación visual y actualizar dependencias
Se agregó una interfaz gráfica con CustomTkinter para que un nuevo usuario pueda buscar películas, calificarlas y obtener recomendaciones mediante BFS y filtrado colaborativo.

También se actualizó el README con las nuevas librerías necesarias, los scripts de interfaz y la configuración de .gitignore.

Co-Authored-By: Andy Condori <196449116+andynary@users.noreply.github.com>
Co-Authored-By: Berna-2024 <182306441+Berna-2024@users.noreply.github.com>
Co-Authored-By: Mittosmc <174610479+Mittosmc@users.noreply.github.com>
Co-Authored-By: JjosephSlater <281017710+JjosephSlater@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/recomendaciones_bfs.xlsx
+++ b/data/recomendaciones_bfs.xlsx
@@ -587,20 +587,20 @@
     <row r="2" ht="35" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>M_128520</t>
+          <t>M_74754</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>The Wedding Ringer (2015)</t>
+          <t>Room, The (2003)</t>
         </is>
       </c>
       <c r="C2" s="9" t="n">
-        <v>2015</v>
+        <v>2003</v>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Comedy</t>
+          <t>Comedy|Drama|Romance</t>
         </is>
       </c>
       <c r="E2" s="11" t="n">
@@ -613,20 +613,20 @@
     <row r="3" ht="35" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>M_69069</t>
+          <t>M_96861</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Fired Up (2009)</t>
+          <t>Taken 2 (2012)</t>
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>2009</v>
+        <v>2012</v>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Comedy</t>
+          <t>Action|Crime|Drama|Thriller</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
@@ -639,20 +639,20 @@
     <row r="4" ht="35" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>M_121231</t>
+          <t>M_6888</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>It Follows (2014)</t>
+          <t>Scary Movie 3 (2003)</t>
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>2014</v>
+        <v>2003</v>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Horror</t>
+          <t>Comedy|Horror</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
@@ -665,20 +665,20 @@
     <row r="5" ht="35" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>M_45668</t>
+          <t>M_69069</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Lake House, The (2006)</t>
+          <t>Fired Up (2009)</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>2006</v>
+        <v>2009</v>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Drama|Fantasy|Romance</t>
+          <t>Comedy</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
@@ -691,20 +691,20 @@
     <row r="6" ht="35" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>M_74754</t>
+          <t>M_87529</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Room, The (2003)</t>
+          <t>Your Highness (2011)</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2003</v>
+        <v>2011</v>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Comedy|Drama|Romance</t>
+          <t>Action|Adventure|Comedy|Fantasy</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
@@ -717,20 +717,20 @@
     <row r="7" ht="35" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>M_96861</t>
+          <t>M_128520</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Taken 2 (2012)</t>
+          <t>The Wedding Ringer (2015)</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>2012</v>
+        <v>2015</v>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Action|Crime|Drama|Thriller</t>
+          <t>Comedy</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
@@ -743,20 +743,20 @@
     <row r="8" ht="35" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>M_6888</t>
+          <t>M_45668</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Scary Movie 3 (2003)</t>
+          <t>Lake House, The (2006)</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>2003</v>
+        <v>2006</v>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Comedy|Horror</t>
+          <t>Drama|Fantasy|Romance</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
@@ -769,20 +769,20 @@
     <row r="9" ht="35" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>M_87529</t>
+          <t>M_121231</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Your Highness (2011)</t>
+          <t>It Follows (2014)</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>2011</v>
+        <v>2014</v>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Action|Adventure|Comedy|Fantasy</t>
+          <t>Horror</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
@@ -795,20 +795,20 @@
     <row r="10" ht="35" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>M_49347</t>
+          <t>M_67788</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Fast Food Nation (2006)</t>
+          <t>Confessions of a Shopaholic (2009)</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>2006</v>
+        <v>2009</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Drama</t>
+          <t>Comedy|Romance</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
@@ -821,16 +821,16 @@
     <row r="11" ht="35" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>M_79428</t>
+          <t>M_87485</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Dinner for Schmucks (2010)</t>
+          <t>Bad Teacher (2011)</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>

</xml_diff>